<commit_message>
Holidays for 2020 and 2021
</commit_message>
<xml_diff>
--- a/data/holidays/holidays.xlsx
+++ b/data/holidays/holidays.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iftek\Documents\MPI\mobility inference\mobility_inference\data\holidays\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40001_{91E5C2EB-3266-4617-B986-3C99A38140E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB8C616E-049E-4E7F-88A6-762B63728A96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="2020 (2)" sheetId="4" r:id="rId1"/>
-    <sheet name="2020" sheetId="1" r:id="rId2"/>
+    <sheet name="2020" sheetId="1" r:id="rId1"/>
+    <sheet name="2021" sheetId="5" r:id="rId2"/>
     <sheet name="2022" sheetId="2" r:id="rId3"/>
-    <sheet name="Tabelle3" sheetId="3" r:id="rId4"/>
+    <sheet name="2020 (2)" sheetId="4" r:id="rId4"/>
+    <sheet name="Comparison" sheetId="3" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="137">
   <si>
     <t>Feiertag</t>
   </si>
@@ -204,12 +205,258 @@
   </si>
   <si>
     <t>Position</t>
+  </si>
+  <si>
+    <t>Wann</t>
+  </si>
+  <si>
+    <t>Neujahr in Deutschland</t>
+  </si>
+  <si>
+    <t>01.01.2020 (Mittwoch)</t>
+  </si>
+  <si>
+    <t>vor 1379 Tagen</t>
+  </si>
+  <si>
+    <t>Heilige Drei Könige</t>
+  </si>
+  <si>
+    <t>06.01.2020 (Montag)</t>
+  </si>
+  <si>
+    <t>Baden-Württemberg, Bayern und Sachsen-Anhalt</t>
+  </si>
+  <si>
+    <t>vor 1374 Tagen</t>
+  </si>
+  <si>
+    <t>08.03.2020 (Sonntag)</t>
+  </si>
+  <si>
+    <t>vor 1312 Tagen</t>
+  </si>
+  <si>
+    <t>10.04.2020 (Freitag)</t>
+  </si>
+  <si>
+    <t>vor 1279 Tagen</t>
+  </si>
+  <si>
+    <t>12.04.2020 (Sonntag)</t>
+  </si>
+  <si>
+    <t>vor 1277 Tagen</t>
+  </si>
+  <si>
+    <t>13.04.2020 (Montag)</t>
+  </si>
+  <si>
+    <t>vor 1276 Tagen</t>
+  </si>
+  <si>
+    <t>vor 1258 Tagen</t>
+  </si>
+  <si>
+    <t>vor 1251 Tagen</t>
+  </si>
+  <si>
+    <t>01.01.2021 (Freitag)</t>
+  </si>
+  <si>
+    <t>vor 1013 Tagen</t>
+  </si>
+  <si>
+    <t>06.01.2021 (Mittwoch)</t>
+  </si>
+  <si>
+    <t>vor 1008 Tagen</t>
+  </si>
+  <si>
+    <t>08.03.2021 (Montag)</t>
+  </si>
+  <si>
+    <t>vor 947 Tagen</t>
+  </si>
+  <si>
+    <t>02.04.2021 (Freitag)</t>
+  </si>
+  <si>
+    <t>vor 922 Tagen</t>
+  </si>
+  <si>
+    <t>04.04.2021 (Sonntag)</t>
+  </si>
+  <si>
+    <t>vor 920 Tagen</t>
+  </si>
+  <si>
+    <t>05.04.2021 (Montag)</t>
+  </si>
+  <si>
+    <t>vor 919 Tagen</t>
+  </si>
+  <si>
+    <t>01.05.2021 (Samstag)</t>
+  </si>
+  <si>
+    <t>vor 893 Tagen</t>
+  </si>
+  <si>
+    <t>13.05.2021 (Donnerstag)</t>
+  </si>
+  <si>
+    <t>vor 881 Tagen</t>
+  </si>
+  <si>
+    <t>Pfingstsonntag in Deutschland</t>
+  </si>
+  <si>
+    <t>(Pfingsten in Deutschland)</t>
+  </si>
+  <si>
+    <t>23.05.2021 (Sonntag)</t>
+  </si>
+  <si>
+    <t>vor 871 Tagen</t>
+  </si>
+  <si>
+    <t>24.05.2021 (Montag)</t>
+  </si>
+  <si>
+    <t>vor 870 Tagen</t>
+  </si>
+  <si>
+    <t>03.06.2021 (Donnerstag)</t>
+  </si>
+  <si>
+    <t>vor 860 Tagen</t>
+  </si>
+  <si>
+    <t>Augsburger Friedensfest </t>
+  </si>
+  <si>
+    <t>08.08.2021 (Sonntag)</t>
+  </si>
+  <si>
+    <t>Bayern</t>
+  </si>
+  <si>
+    <t>vor 794 Tagen</t>
+  </si>
+  <si>
+    <t>15.08.2021 (Sonntag)</t>
+  </si>
+  <si>
+    <t>vor 787 Tagen</t>
+  </si>
+  <si>
+    <t>20.09.2021 (Montag)</t>
+  </si>
+  <si>
+    <t>vor 751 Tagen</t>
+  </si>
+  <si>
+    <t>03.10.2021 (Sonntag)</t>
+  </si>
+  <si>
+    <t>vor 738 Tagen</t>
+  </si>
+  <si>
+    <t>31.10.2021 (Sonntag)</t>
+  </si>
+  <si>
+    <t>vor 710 Tagen</t>
+  </si>
+  <si>
+    <t>01.11.2021 (Montag)</t>
+  </si>
+  <si>
+    <t>vor 709 Tagen</t>
+  </si>
+  <si>
+    <t>17.11.2021 (Mittwoch)</t>
+  </si>
+  <si>
+    <t>vor 693 Tagen</t>
+  </si>
+  <si>
+    <t>1. Weihnachtstag in Deutschland</t>
+  </si>
+  <si>
+    <t>(Weihnachten in Deutschland)</t>
+  </si>
+  <si>
+    <t>25.12.2021 (Samstag)</t>
+  </si>
+  <si>
+    <t>vor 655 Tagen</t>
+  </si>
+  <si>
+    <t>2. Weihnachtstag in Deutschland</t>
+  </si>
+  <si>
+    <t>26.12.2021 (Sonntag)</t>
+  </si>
+  <si>
+    <t>vor 654 Tagen</t>
+  </si>
+  <si>
+    <t>vor 1238 Tagen</t>
+  </si>
+  <si>
+    <t>31.05.2020 (Sonntag)</t>
+  </si>
+  <si>
+    <t>vor 1228 Tagen</t>
+  </si>
+  <si>
+    <t>vor 1227 Tagen</t>
+  </si>
+  <si>
+    <t>vor 1217 Tagen</t>
+  </si>
+  <si>
+    <t>08.08.2020 (Samstag)</t>
+  </si>
+  <si>
+    <t>vor 1159 Tagen</t>
+  </si>
+  <si>
+    <t>vor 1152 Tagen</t>
+  </si>
+  <si>
+    <t>vor 1116 Tagen</t>
+  </si>
+  <si>
+    <t>vor 1103 Tagen</t>
+  </si>
+  <si>
+    <t>vor 1075 Tagen</t>
+  </si>
+  <si>
+    <t>vor 1074 Tagen</t>
+  </si>
+  <si>
+    <t>vor 1057 Tagen</t>
+  </si>
+  <si>
+    <t>25.12.2020 (Freitag)</t>
+  </si>
+  <si>
+    <t>vor 1020 Tagen</t>
+  </si>
+  <si>
+    <t>26.12.2020 (Samstag)</t>
+  </si>
+  <si>
+    <t>vor 1019 Tagen</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="6">
     <font>
       <sz val="11"/>
@@ -314,7 +561,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -350,30 +597,6 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -385,6 +608,45 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -699,238 +961,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
-  <cols>
-    <col min="3" max="3" width="13" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" ht="15" thickBot="1">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1">
-        <v>2020</v>
-      </c>
-      <c r="E1">
-        <v>2022</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" s="25" customFormat="1" ht="43.8" thickBot="1">
-      <c r="A2" s="22" t="s">
-        <v>11</v>
-      </c>
-      <c r="B2" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" s="23" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="24">
-        <v>6</v>
-      </c>
-      <c r="E2" s="24">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" s="25" customFormat="1" ht="43.8" thickBot="1">
-      <c r="A3" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="B3" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" s="23" t="s">
-        <v>4</v>
-      </c>
-      <c r="D3" s="24">
-        <v>7</v>
-      </c>
-      <c r="E3" s="25">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="58.2" thickBot="1">
-      <c r="A4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="5">
-        <v>9</v>
-      </c>
-      <c r="E4" s="9">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="43.8" thickBot="1">
-      <c r="A5" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="5">
-        <v>11</v>
-      </c>
-      <c r="E5" s="9">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="80.400000000000006" thickBot="1">
-      <c r="A6" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" s="9">
-        <v>12</v>
-      </c>
-      <c r="E6" s="5">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="58.2" thickBot="1">
-      <c r="A7" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="D7" s="9">
-        <v>21</v>
-      </c>
-      <c r="E7" s="5">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="43.8" thickBot="1">
-      <c r="A8" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="D8" s="5">
-        <v>26</v>
-      </c>
-      <c r="E8" s="9">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="43.8" thickBot="1">
-      <c r="A9" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" s="9">
-        <v>28</v>
-      </c>
-      <c r="E9" s="5">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="126" thickBot="1">
-      <c r="A10" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="D10" s="5">
-        <v>32</v>
-      </c>
-      <c r="E10" s="9">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="80.400000000000006" thickBot="1">
-      <c r="A11" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="D11" s="9">
-        <v>32</v>
-      </c>
-      <c r="E11" s="5">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" s="25" customFormat="1" ht="43.2">
-      <c r="A12" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="B12" s="23" t="s">
-        <v>37</v>
-      </c>
-      <c r="C12" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="D12" s="25">
-        <v>35</v>
-      </c>
-      <c r="E12" s="25">
-        <v>34</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" display="https://www.ferienwiki.de/feiertage/tag-der-arbeit"/>
-    <hyperlink ref="A3" r:id="rId2" display="https://www.ferienwiki.de/feiertage/tag-der-befreiung"/>
-    <hyperlink ref="A4" r:id="rId3" display="https://www.ferienwiki.de/feiertage/christi-himmelfahrt"/>
-    <hyperlink ref="A5" r:id="rId4" display="https://www.ferienwiki.de/feiertage/pfingstmontag"/>
-    <hyperlink ref="A6" r:id="rId5" display="https://www.ferienwiki.de/feiertage/fronleichnam"/>
-    <hyperlink ref="A7" r:id="rId6" display="https://www.ferienwiki.de/feiertage/maria-himmelfahrt"/>
-    <hyperlink ref="A8" r:id="rId7" display="https://www.ferienwiki.de/feiertage/weltkindertag"/>
-    <hyperlink ref="A9" r:id="rId8" display="https://www.ferienwiki.de/feiertage/tag-der-deutschen-einheit"/>
-    <hyperlink ref="A10" r:id="rId9" display="https://www.ferienwiki.de/feiertage/reformationstag"/>
-    <hyperlink ref="A11" r:id="rId10" display="https://www.ferienwiki.de/feiertage/allerheiligen"/>
-    <hyperlink ref="A12" r:id="rId11" display="https://www.ferienwiki.de/feiertage/buss-und-bettag"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D12"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
     <col min="3" max="3" width="13" customWidth="1"/>
@@ -946,181 +978,835 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="43.8" thickBot="1">
+      <c r="D1" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="29.4" thickBot="1">
       <c r="A2" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="46.2" thickBot="1">
+      <c r="A3" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="29.4" thickBot="1">
+      <c r="A4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="14.4" customHeight="1">
+      <c r="A5" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="20" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="29.4" thickBot="1">
+      <c r="A6" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="19"/>
+      <c r="C6" s="19"/>
+      <c r="D6" s="21"/>
+    </row>
+    <row r="7" spans="1:4" ht="14.4" customHeight="1">
+      <c r="A7" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="22" t="s">
+        <v>67</v>
+      </c>
+      <c r="C7" s="22" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="24" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="29.4" thickBot="1">
+      <c r="A8" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="23"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="25"/>
+    </row>
+    <row r="9" spans="1:4" ht="43.2">
+      <c r="A9" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="20" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="29.4" thickBot="1">
+      <c r="A10" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="19"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="21"/>
+    </row>
+    <row r="11" spans="1:4" ht="43.8" thickBot="1">
+      <c r="A11" s="3" t="s">
         <v>11</v>
       </c>
+      <c r="B11" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="43.8" thickBot="1">
+      <c r="A12" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="58.2" thickBot="1">
+      <c r="A13" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="43.2">
+      <c r="A14" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="B14" s="18" t="s">
+        <v>121</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" s="20" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="29.4" thickBot="1">
+      <c r="A15" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="B15" s="19"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="21"/>
+    </row>
+    <row r="16" spans="1:4" ht="43.2">
+      <c r="A16" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="D16" s="24" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="29.4" thickBot="1">
+      <c r="A17" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="B17" s="23"/>
+      <c r="C17" s="23"/>
+      <c r="D17" s="25"/>
+    </row>
+    <row r="18" spans="1:4" ht="80.400000000000006" thickBot="1">
+      <c r="A18" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="29.4" thickBot="1">
+      <c r="A19" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="58.2" thickBot="1">
+      <c r="A20" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="43.8" thickBot="1">
+      <c r="A21" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="43.8" thickBot="1">
+      <c r="A22" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="126" thickBot="1">
+      <c r="A23" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="80.400000000000006" thickBot="1">
+      <c r="A24" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="43.8" thickBot="1">
+      <c r="A25" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="57.6">
+      <c r="A26" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="B26" s="18" t="s">
+        <v>133</v>
+      </c>
+      <c r="C26" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="D26" s="20" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="43.8" thickBot="1">
+      <c r="A27" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="B27" s="19"/>
+      <c r="C27" s="19"/>
+      <c r="D27" s="21"/>
+    </row>
+    <row r="28" spans="1:4" ht="57.6">
+      <c r="A28" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="B28" s="27" t="s">
+        <v>135</v>
+      </c>
+      <c r="C28" s="27" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28" s="29" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="43.2">
+      <c r="A29" s="26" t="s">
+        <v>114</v>
+      </c>
+      <c r="B29" s="28"/>
+      <c r="C29" s="28"/>
+      <c r="D29" s="30"/>
+    </row>
+  </sheetData>
+  <mergeCells count="21">
+    <mergeCell ref="B28:B29"/>
+    <mergeCell ref="C28:C29"/>
+    <mergeCell ref="D28:D29"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="C16:C17"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="D26:D27"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" display="https://www.ferienwiki.de/feiertage/neujahr" xr:uid="{7DE2B16C-C511-4A8D-8C33-6F429FF8F0F6}"/>
+    <hyperlink ref="A3" r:id="rId2" display="https://www.ferienwiki.de/feiertage/heilige-drei-koenige" xr:uid="{11F209A1-B86D-4917-BCB1-32208C24AADD}"/>
+    <hyperlink ref="A4" r:id="rId3" display="https://www.ferienwiki.de/feiertage/internationaler-frauentag" xr:uid="{9C5A6F07-EC21-4E19-97B7-3D9ADD478A38}"/>
+    <hyperlink ref="A5" r:id="rId4" display="https://www.ferienwiki.de/feiertage/karfreitag" xr:uid="{0ACA7EE1-0D80-492B-B052-642CE8D6C719}"/>
+    <hyperlink ref="A6" r:id="rId5" display="https://www.ferienwiki.de/feiertagsperioden/ostern" xr:uid="{948705E5-ACE3-46BB-A0D3-A9609A0C56C6}"/>
+    <hyperlink ref="A7" r:id="rId6" display="https://www.ferienwiki.de/feiertage/ostersonntag" xr:uid="{E125486D-220C-487E-A014-E6C1E7771F3D}"/>
+    <hyperlink ref="A8" r:id="rId7" display="https://www.ferienwiki.de/feiertagsperioden/ostern" xr:uid="{C4EDE9B4-1BBE-4270-B3CA-FE469D36753B}"/>
+    <hyperlink ref="A9" r:id="rId8" display="https://www.ferienwiki.de/feiertage/ostermontag" xr:uid="{667883A6-FB67-4E21-A07D-0F647D527B0E}"/>
+    <hyperlink ref="A10" r:id="rId9" display="https://www.ferienwiki.de/feiertagsperioden/ostern" xr:uid="{0F58E781-0727-44F1-8F7A-9BE53166973B}"/>
+    <hyperlink ref="A11" r:id="rId10" display="https://www.ferienwiki.de/feiertage/tag-der-arbeit" xr:uid="{7AC97179-583C-4935-B7CB-601E4ABF1666}"/>
+    <hyperlink ref="A12" r:id="rId11" display="https://www.ferienwiki.de/feiertage/tag-der-befreiung" xr:uid="{29F9CEF2-98C9-42CF-A272-E9B21F07279B}"/>
+    <hyperlink ref="A13" r:id="rId12" display="https://www.ferienwiki.de/feiertage/christi-himmelfahrt" xr:uid="{8BBD2E3B-84A1-4B23-ABCE-F0A6F5D0C3F1}"/>
+    <hyperlink ref="A14" r:id="rId13" display="https://www.ferienwiki.de/feiertage/pfingstsonntag" xr:uid="{AA2CA971-EAA6-4F0D-A14D-D3764010D32A}"/>
+    <hyperlink ref="A15" r:id="rId14" display="https://www.ferienwiki.de/feiertagsperioden/pfingsten" xr:uid="{763CEAD3-5D99-4D2F-B633-1DE890B38D7A}"/>
+    <hyperlink ref="A16" r:id="rId15" display="https://www.ferienwiki.de/feiertage/pfingstmontag" xr:uid="{B5360A05-012F-4766-A6D5-4DA5A22F9CAB}"/>
+    <hyperlink ref="A17" r:id="rId16" display="https://www.ferienwiki.de/feiertagsperioden/pfingsten" xr:uid="{EC88AB5B-187B-4322-909D-84479E0F7C0B}"/>
+    <hyperlink ref="A18" r:id="rId17" display="https://www.ferienwiki.de/feiertage/fronleichnam" xr:uid="{54B1B0FF-0931-4705-B3F1-39B8F77E7803}"/>
+    <hyperlink ref="A19" r:id="rId18" display="https://www.ferienwiki.de/feiertage/augsburger-friedensfest" xr:uid="{BE08834C-7F78-4008-A9B2-2360BCA230B7}"/>
+    <hyperlink ref="A20" r:id="rId19" display="https://www.ferienwiki.de/feiertage/maria-himmelfahrt" xr:uid="{07631940-5638-44E9-9564-9E654142F5B6}"/>
+    <hyperlink ref="A21" r:id="rId20" display="https://www.ferienwiki.de/feiertage/weltkindertag" xr:uid="{79F7F8D7-E99A-4827-96CF-1CEB163D9662}"/>
+    <hyperlink ref="A22" r:id="rId21" display="https://www.ferienwiki.de/feiertage/tag-der-deutschen-einheit" xr:uid="{055C468F-6D9D-4ED1-BE68-CEF9776115F3}"/>
+    <hyperlink ref="A23" r:id="rId22" display="https://www.ferienwiki.de/feiertage/reformationstag" xr:uid="{AF5F9774-E7F1-4C45-A178-7BE4238B6FE4}"/>
+    <hyperlink ref="A24" r:id="rId23" display="https://www.ferienwiki.de/feiertage/allerheiligen" xr:uid="{952313B1-E0A1-430D-A639-1A9E34085478}"/>
+    <hyperlink ref="A25" r:id="rId24" display="https://www.ferienwiki.de/feiertage/buss-und-bettag" xr:uid="{E9CE8BC4-EC9D-4336-823E-D61E8628B4CE}"/>
+    <hyperlink ref="A26" r:id="rId25" display="https://www.ferienwiki.de/feiertage/erster-weihnachtstag" xr:uid="{2DE21E74-6F99-4CBB-B850-C528B15B38F3}"/>
+    <hyperlink ref="A27" r:id="rId26" display="https://www.ferienwiki.de/feiertagsperioden/weihnachten" xr:uid="{DEE94E00-4A43-4690-978A-8D54EF258376}"/>
+    <hyperlink ref="A28" r:id="rId27" display="https://www.ferienwiki.de/feiertage/zweiter-weihnachtstag" xr:uid="{B1440C08-578B-432E-846A-E1B5EFA03D9D}"/>
+    <hyperlink ref="A29" r:id="rId28" display="https://www.ferienwiki.de/feiertagsperioden/weihnachten" xr:uid="{2D42EBF2-2B4A-4F22-9E47-3E5974742B2C}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C129FF9-E05F-4030-AAE3-14651069BC65}">
+  <dimension ref="A1:D28"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="3" max="3" width="13.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="25.2" thickBot="1">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="29.4" thickBot="1">
+      <c r="A2" s="3" t="s">
+        <v>56</v>
+      </c>
       <c r="B2" s="4" t="s">
-        <v>12</v>
+        <v>73</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="5">
+      <c r="D2" s="5" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="57.6" thickBot="1">
+      <c r="A3" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="29.4" thickBot="1">
+      <c r="A4" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="28.8">
+      <c r="A5" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="20" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="29.4" thickBot="1">
+      <c r="A6" s="6" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="43.8" thickBot="1">
-      <c r="A3" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="D3" s="9">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="58.2" thickBot="1">
-      <c r="A4" s="3" t="s">
+      <c r="B6" s="19"/>
+      <c r="C6" s="19"/>
+      <c r="D6" s="21"/>
+    </row>
+    <row r="7" spans="1:4" ht="43.2">
+      <c r="A7" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="22" t="s">
+        <v>81</v>
+      </c>
+      <c r="C7" s="22" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="24" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="29.4" thickBot="1">
+      <c r="A8" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="23"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="25"/>
+    </row>
+    <row r="9" spans="1:4" ht="43.2">
+      <c r="A9" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="20" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="29.4" thickBot="1">
+      <c r="A10" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="19"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="21"/>
+    </row>
+    <row r="11" spans="1:4" ht="43.8" thickBot="1">
+      <c r="A11" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="58.2" thickBot="1">
+      <c r="A12" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="5">
+      <c r="B12" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="43.2">
+      <c r="A13" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B13" s="22" t="s">
+        <v>91</v>
+      </c>
+      <c r="C13" s="22" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="43.8" thickBot="1">
-      <c r="A5" s="3" t="s">
+      <c r="D13" s="24" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="29.4" thickBot="1">
+      <c r="A14" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="B14" s="23"/>
+      <c r="C14" s="23"/>
+      <c r="D14" s="25"/>
+    </row>
+    <row r="15" spans="1:4" ht="43.2">
+      <c r="A15" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D5" s="5">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="80.400000000000006" thickBot="1">
-      <c r="A6" s="7" t="s">
+      <c r="B15" s="18" t="s">
+        <v>93</v>
+      </c>
+      <c r="C15" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="D15" s="20" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="29.4" thickBot="1">
+      <c r="A16" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="B16" s="19"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="21"/>
+    </row>
+    <row r="17" spans="1:4" ht="103.2" thickBot="1">
+      <c r="A17" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C6" s="8" t="s">
+      <c r="B17" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C17" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="9">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="58.2" thickBot="1">
-      <c r="A7" s="7" t="s">
+      <c r="D17" s="5" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="29.4" thickBot="1">
+      <c r="A18" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="58.2" thickBot="1">
+      <c r="A19" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" s="8" t="s">
+      <c r="B19" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C19" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="9">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" thickBot="1">
-      <c r="A8" s="3" t="s">
+      <c r="D19" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="43.8" thickBot="1">
+      <c r="A20" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C8" s="4" t="s">
+      <c r="B20" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="C20" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="D8" s="5">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" thickBot="1">
-      <c r="A9" s="7" t="s">
+      <c r="D20" s="9" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="43.8" thickBot="1">
+      <c r="A21" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="8" t="s">
-        <v>29</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="D9" s="9">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="126" thickBot="1">
-      <c r="A10" s="3" t="s">
+      <c r="B21" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="137.4" thickBot="1">
+      <c r="A22" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C10" s="4" t="s">
+      <c r="B22" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="C22" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="D10" s="5">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="80.400000000000006" thickBot="1">
-      <c r="A11" s="7" t="s">
+      <c r="D22" s="9" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="91.8" thickBot="1">
+      <c r="A23" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B11" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="C11" s="8" t="s">
+      <c r="B23" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="C23" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D11" s="9">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="43.2">
-      <c r="A12" s="11" t="s">
+      <c r="D23" s="5" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="43.8" thickBot="1">
+      <c r="A24" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="C12" s="12" t="s">
+      <c r="B24" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="C24" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="D12" s="1">
-        <v>35</v>
-      </c>
+      <c r="D24" s="9" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="57.6">
+      <c r="A25" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="B25" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="C25" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="D25" s="24" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="43.8" thickBot="1">
+      <c r="A26" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="B26" s="23"/>
+      <c r="C26" s="23"/>
+      <c r="D26" s="25"/>
+    </row>
+    <row r="27" spans="1:4" ht="57.6">
+      <c r="A27" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="B27" s="27" t="s">
+        <v>118</v>
+      </c>
+      <c r="C27" s="27" t="s">
+        <v>7</v>
+      </c>
+      <c r="D27" s="29" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="43.2">
+      <c r="A28" s="26" t="s">
+        <v>114</v>
+      </c>
+      <c r="B28" s="28"/>
+      <c r="C28" s="28"/>
+      <c r="D28" s="30"/>
     </row>
   </sheetData>
+  <mergeCells count="21">
+    <mergeCell ref="B27:B28"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="D27:D28"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+  </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" display="https://www.ferienwiki.de/feiertage/tag-der-arbeit"/>
-    <hyperlink ref="A3" r:id="rId2" display="https://www.ferienwiki.de/feiertage/tag-der-befreiung"/>
-    <hyperlink ref="A4" r:id="rId3" display="https://www.ferienwiki.de/feiertage/christi-himmelfahrt"/>
-    <hyperlink ref="A5" r:id="rId4" display="https://www.ferienwiki.de/feiertage/pfingstmontag"/>
-    <hyperlink ref="A6" r:id="rId5" display="https://www.ferienwiki.de/feiertage/fronleichnam"/>
-    <hyperlink ref="A7" r:id="rId6" display="https://www.ferienwiki.de/feiertage/maria-himmelfahrt"/>
-    <hyperlink ref="A8" r:id="rId7" display="https://www.ferienwiki.de/feiertage/weltkindertag"/>
-    <hyperlink ref="A9" r:id="rId8" display="https://www.ferienwiki.de/feiertage/tag-der-deutschen-einheit"/>
-    <hyperlink ref="A10" r:id="rId9" display="https://www.ferienwiki.de/feiertage/reformationstag"/>
-    <hyperlink ref="A11" r:id="rId10" display="https://www.ferienwiki.de/feiertage/allerheiligen"/>
-    <hyperlink ref="A12" r:id="rId11" display="https://www.ferienwiki.de/feiertage/buss-und-bettag"/>
+    <hyperlink ref="A2" r:id="rId1" display="https://www.ferienwiki.de/feiertage/neujahr" xr:uid="{AD790FF0-3189-476B-9EEB-9B5F84A9F580}"/>
+    <hyperlink ref="A3" r:id="rId2" display="https://www.ferienwiki.de/feiertage/heilige-drei-koenige" xr:uid="{60406553-45CA-404F-B502-91F895B3E249}"/>
+    <hyperlink ref="A4" r:id="rId3" display="https://www.ferienwiki.de/feiertage/internationaler-frauentag" xr:uid="{D20468FA-5D3F-4B14-8445-3692738D9AA4}"/>
+    <hyperlink ref="A5" r:id="rId4" display="https://www.ferienwiki.de/feiertage/karfreitag" xr:uid="{E42B0CD2-C6ED-4F59-99B8-F788D825680B}"/>
+    <hyperlink ref="A6" r:id="rId5" display="https://www.ferienwiki.de/feiertagsperioden/ostern" xr:uid="{D4F2D9F2-9E85-49EA-BDE2-E54E4245FEC8}"/>
+    <hyperlink ref="A7" r:id="rId6" display="https://www.ferienwiki.de/feiertage/ostersonntag" xr:uid="{B83C7C3D-0F0F-4074-8298-A2C1FE03E69B}"/>
+    <hyperlink ref="A8" r:id="rId7" display="https://www.ferienwiki.de/feiertagsperioden/ostern" xr:uid="{8220E177-715F-4DBD-96F1-015FBF44CD4C}"/>
+    <hyperlink ref="A9" r:id="rId8" display="https://www.ferienwiki.de/feiertage/ostermontag" xr:uid="{8FAA659C-0DA1-4961-AA4E-B98A90827851}"/>
+    <hyperlink ref="A10" r:id="rId9" display="https://www.ferienwiki.de/feiertagsperioden/ostern" xr:uid="{2513DB33-A7E1-4AF3-8B4B-CAA247A5BE53}"/>
+    <hyperlink ref="A11" r:id="rId10" display="https://www.ferienwiki.de/feiertage/tag-der-arbeit" xr:uid="{F015C5C8-62C3-45E1-B2D3-5B19CE70B526}"/>
+    <hyperlink ref="A12" r:id="rId11" display="https://www.ferienwiki.de/feiertage/christi-himmelfahrt" xr:uid="{D7C67A63-1FA4-4C6E-A639-72A150F88DE7}"/>
+    <hyperlink ref="A13" r:id="rId12" display="https://www.ferienwiki.de/feiertage/pfingstsonntag" xr:uid="{696BB143-A006-42FA-8AE9-841E8036110D}"/>
+    <hyperlink ref="A14" r:id="rId13" display="https://www.ferienwiki.de/feiertagsperioden/pfingsten" xr:uid="{0BFC5F0F-D781-420C-AF52-804C80B0C4F9}"/>
+    <hyperlink ref="A15" r:id="rId14" display="https://www.ferienwiki.de/feiertage/pfingstmontag" xr:uid="{8C87104F-370C-4681-8C22-FEE7EB4DCB09}"/>
+    <hyperlink ref="A16" r:id="rId15" display="https://www.ferienwiki.de/feiertagsperioden/pfingsten" xr:uid="{90562100-0867-4785-8059-E12AB1B82CB3}"/>
+    <hyperlink ref="A17" r:id="rId16" display="https://www.ferienwiki.de/feiertage/fronleichnam" xr:uid="{6A2FBD75-A99A-4D16-B7DF-A4A00700C386}"/>
+    <hyperlink ref="A18" r:id="rId17" display="https://www.ferienwiki.de/feiertage/augsburger-friedensfest" xr:uid="{B99D07B5-8FC4-4ED3-956A-4E04EA353D2C}"/>
+    <hyperlink ref="A19" r:id="rId18" display="https://www.ferienwiki.de/feiertage/maria-himmelfahrt" xr:uid="{603C42C2-20EC-4FF0-A43E-AF34330AA843}"/>
+    <hyperlink ref="A20" r:id="rId19" display="https://www.ferienwiki.de/feiertage/weltkindertag" xr:uid="{07320D33-926F-49D7-913B-20655B1D1828}"/>
+    <hyperlink ref="A21" r:id="rId20" display="https://www.ferienwiki.de/feiertage/tag-der-deutschen-einheit" xr:uid="{FF9D6F22-70FA-4911-8CC4-7CDDF9572BE7}"/>
+    <hyperlink ref="A22" r:id="rId21" display="https://www.ferienwiki.de/feiertage/reformationstag" xr:uid="{856D5BFA-7DCA-4584-A44E-AD19BA8BA310}"/>
+    <hyperlink ref="A23" r:id="rId22" display="https://www.ferienwiki.de/feiertage/allerheiligen" xr:uid="{95ECDFD0-2634-4A97-8259-71BF0860B217}"/>
+    <hyperlink ref="A24" r:id="rId23" display="https://www.ferienwiki.de/feiertage/buss-und-bettag" xr:uid="{0AD440F9-4090-4524-88EF-B552FA130E67}"/>
+    <hyperlink ref="A25" r:id="rId24" display="https://www.ferienwiki.de/feiertage/erster-weihnachtstag" xr:uid="{E90B71A2-8F73-485A-9006-15E77E2C87CE}"/>
+    <hyperlink ref="A26" r:id="rId25" display="https://www.ferienwiki.de/feiertagsperioden/weihnachten" xr:uid="{7B3F5E40-E357-4563-8DBC-565074AE1E58}"/>
+    <hyperlink ref="A27" r:id="rId26" display="https://www.ferienwiki.de/feiertage/zweiter-weihnachtstag" xr:uid="{61FF5E70-4F25-42AA-88CB-2822A6D5F5A9}"/>
+    <hyperlink ref="A28" r:id="rId27" display="https://www.ferienwiki.de/feiertagsperioden/weihnachten" xr:uid="{EB972D06-424F-4652-A56E-B5A90B0FFCF2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
@@ -1137,7 +1823,7 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="21" t="s">
+      <c r="D1" s="13" t="s">
         <v>54</v>
       </c>
     </row>
@@ -1157,61 +1843,61 @@
       <c r="A3" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="15"/>
+      <c r="C3" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="20"/>
     </row>
     <row r="4" spans="1:4" ht="29.4" thickBot="1">
       <c r="A4" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="14"/>
-      <c r="C4" s="14"/>
-      <c r="D4" s="16"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="21"/>
     </row>
     <row r="5" spans="1:4" ht="43.2">
       <c r="A5" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="C5" s="17" t="s">
+      <c r="C5" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="19"/>
+      <c r="D5" s="24"/>
     </row>
     <row r="6" spans="1:4" ht="29.4" thickBot="1">
       <c r="A6" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="18"/>
-      <c r="C6" s="18"/>
-      <c r="D6" s="20"/>
+      <c r="B6" s="23"/>
+      <c r="C6" s="23"/>
+      <c r="D6" s="25"/>
     </row>
     <row r="7" spans="1:4" ht="43.2">
       <c r="A7" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B7" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="C7" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7" s="15"/>
+      <c r="C7" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="20"/>
     </row>
     <row r="8" spans="1:4" ht="29.4" thickBot="1">
       <c r="A8" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="16"/>
+      <c r="B8" s="19"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="21"/>
     </row>
     <row r="9" spans="1:4" ht="43.8" thickBot="1">
       <c r="A9" s="3" t="s">
@@ -1311,7 +1997,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="16" spans="1:4" thickBot="1">
+    <row r="16" spans="1:4" ht="126" thickBot="1">
       <c r="A16" s="7" t="s">
         <v>30</v>
       </c>
@@ -1366,30 +2052,260 @@
     <mergeCell ref="D5:D6"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" display="https://www.ferienwiki.de/feiertage/internationaler-frauentag"/>
-    <hyperlink ref="A3" r:id="rId2" display="https://www.ferienwiki.de/feiertage/karfreitag"/>
-    <hyperlink ref="A4" r:id="rId3" display="https://www.ferienwiki.de/feiertagsperioden/ostern"/>
-    <hyperlink ref="A5" r:id="rId4" display="https://www.ferienwiki.de/feiertage/ostersonntag"/>
-    <hyperlink ref="A6" r:id="rId5" display="https://www.ferienwiki.de/feiertagsperioden/ostern"/>
-    <hyperlink ref="A7" r:id="rId6" display="https://www.ferienwiki.de/feiertage/ostermontag"/>
-    <hyperlink ref="A8" r:id="rId7" display="https://www.ferienwiki.de/feiertagsperioden/ostern"/>
-    <hyperlink ref="A9" r:id="rId8" display="https://www.ferienwiki.de/feiertage/tag-der-arbeit"/>
-    <hyperlink ref="A10" r:id="rId9" display="https://www.ferienwiki.de/feiertage/christi-himmelfahrt"/>
-    <hyperlink ref="A11" r:id="rId10" display="https://www.ferienwiki.de/feiertage/pfingstmontag"/>
-    <hyperlink ref="A12" r:id="rId11" display="https://www.ferienwiki.de/feiertage/fronleichnam"/>
-    <hyperlink ref="A13" r:id="rId12" display="https://www.ferienwiki.de/feiertage/maria-himmelfahrt"/>
-    <hyperlink ref="A14" r:id="rId13" display="https://www.ferienwiki.de/feiertage/weltkindertag"/>
-    <hyperlink ref="A15" r:id="rId14" display="https://www.ferienwiki.de/feiertage/tag-der-deutschen-einheit"/>
-    <hyperlink ref="A16" r:id="rId15" display="https://www.ferienwiki.de/feiertage/reformationstag"/>
-    <hyperlink ref="A17" r:id="rId16" display="https://www.ferienwiki.de/feiertage/allerheiligen"/>
-    <hyperlink ref="A18" r:id="rId17" display="https://www.ferienwiki.de/feiertage/buss-und-bettag"/>
+    <hyperlink ref="A2" r:id="rId1" display="https://www.ferienwiki.de/feiertage/internationaler-frauentag" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
+    <hyperlink ref="A3" r:id="rId2" display="https://www.ferienwiki.de/feiertage/karfreitag" xr:uid="{00000000-0004-0000-0200-000001000000}"/>
+    <hyperlink ref="A4" r:id="rId3" display="https://www.ferienwiki.de/feiertagsperioden/ostern" xr:uid="{00000000-0004-0000-0200-000002000000}"/>
+    <hyperlink ref="A5" r:id="rId4" display="https://www.ferienwiki.de/feiertage/ostersonntag" xr:uid="{00000000-0004-0000-0200-000003000000}"/>
+    <hyperlink ref="A6" r:id="rId5" display="https://www.ferienwiki.de/feiertagsperioden/ostern" xr:uid="{00000000-0004-0000-0200-000004000000}"/>
+    <hyperlink ref="A7" r:id="rId6" display="https://www.ferienwiki.de/feiertage/ostermontag" xr:uid="{00000000-0004-0000-0200-000005000000}"/>
+    <hyperlink ref="A8" r:id="rId7" display="https://www.ferienwiki.de/feiertagsperioden/ostern" xr:uid="{00000000-0004-0000-0200-000006000000}"/>
+    <hyperlink ref="A9" r:id="rId8" display="https://www.ferienwiki.de/feiertage/tag-der-arbeit" xr:uid="{00000000-0004-0000-0200-000007000000}"/>
+    <hyperlink ref="A10" r:id="rId9" display="https://www.ferienwiki.de/feiertage/christi-himmelfahrt" xr:uid="{00000000-0004-0000-0200-000008000000}"/>
+    <hyperlink ref="A11" r:id="rId10" display="https://www.ferienwiki.de/feiertage/pfingstmontag" xr:uid="{00000000-0004-0000-0200-000009000000}"/>
+    <hyperlink ref="A12" r:id="rId11" display="https://www.ferienwiki.de/feiertage/fronleichnam" xr:uid="{00000000-0004-0000-0200-00000A000000}"/>
+    <hyperlink ref="A13" r:id="rId12" display="https://www.ferienwiki.de/feiertage/maria-himmelfahrt" xr:uid="{00000000-0004-0000-0200-00000B000000}"/>
+    <hyperlink ref="A14" r:id="rId13" display="https://www.ferienwiki.de/feiertage/weltkindertag" xr:uid="{00000000-0004-0000-0200-00000C000000}"/>
+    <hyperlink ref="A15" r:id="rId14" display="https://www.ferienwiki.de/feiertage/tag-der-deutschen-einheit" xr:uid="{00000000-0004-0000-0200-00000D000000}"/>
+    <hyperlink ref="A16" r:id="rId15" display="https://www.ferienwiki.de/feiertage/reformationstag" xr:uid="{00000000-0004-0000-0200-00000E000000}"/>
+    <hyperlink ref="A17" r:id="rId16" display="https://www.ferienwiki.de/feiertage/allerheiligen" xr:uid="{00000000-0004-0000-0200-00000F000000}"/>
+    <hyperlink ref="A18" r:id="rId17" display="https://www.ferienwiki.de/feiertage/buss-und-bettag" xr:uid="{00000000-0004-0000-0200-000010000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
+  <cols>
+    <col min="3" max="3" width="13" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="15" thickBot="1">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1">
+        <v>2020</v>
+      </c>
+      <c r="E1">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" s="17" customFormat="1" ht="43.8" thickBot="1">
+      <c r="A2" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="16">
+        <v>6</v>
+      </c>
+      <c r="E2" s="16">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" s="17" customFormat="1" ht="43.8" thickBot="1">
+      <c r="A3" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="16">
+        <v>7</v>
+      </c>
+      <c r="E3" s="17">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="58.2" thickBot="1">
+      <c r="A4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="5">
+        <v>9</v>
+      </c>
+      <c r="E4" s="9">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="43.8" thickBot="1">
+      <c r="A5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5">
+        <v>11</v>
+      </c>
+      <c r="E5" s="9">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="80.400000000000006" thickBot="1">
+      <c r="A6" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="9">
+        <v>12</v>
+      </c>
+      <c r="E6" s="5">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="58.2" thickBot="1">
+      <c r="A7" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="9">
+        <v>21</v>
+      </c>
+      <c r="E7" s="5">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="43.8" thickBot="1">
+      <c r="A8" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="5">
+        <v>26</v>
+      </c>
+      <c r="E8" s="9">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="43.8" thickBot="1">
+      <c r="A9" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="9">
+        <v>28</v>
+      </c>
+      <c r="E9" s="5">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="126" thickBot="1">
+      <c r="A10" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D10" s="5">
+        <v>32</v>
+      </c>
+      <c r="E10" s="9">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="80.400000000000006" thickBot="1">
+      <c r="A11" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" s="9">
+        <v>32</v>
+      </c>
+      <c r="E11" s="5">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" s="17" customFormat="1" ht="43.2">
+      <c r="A12" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="C12" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" s="17">
+        <v>35</v>
+      </c>
+      <c r="E12" s="17">
+        <v>34</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" display="https://www.ferienwiki.de/feiertage/tag-der-arbeit" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="A3" r:id="rId2" display="https://www.ferienwiki.de/feiertage/tag-der-befreiung" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="A4" r:id="rId3" display="https://www.ferienwiki.de/feiertage/christi-himmelfahrt" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="A5" r:id="rId4" display="https://www.ferienwiki.de/feiertage/pfingstmontag" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="A6" r:id="rId5" display="https://www.ferienwiki.de/feiertage/fronleichnam" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="A7" r:id="rId6" display="https://www.ferienwiki.de/feiertage/maria-himmelfahrt" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="A8" r:id="rId7" display="https://www.ferienwiki.de/feiertage/weltkindertag" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="A9" r:id="rId8" display="https://www.ferienwiki.de/feiertage/tag-der-deutschen-einheit" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="A10" r:id="rId9" display="https://www.ferienwiki.de/feiertage/reformationstag" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="A11" r:id="rId10" display="https://www.ferienwiki.de/feiertage/allerheiligen" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="A12" r:id="rId11" display="https://www.ferienwiki.de/feiertage/buss-und-bettag" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
@@ -1397,10 +2313,10 @@
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="21">
+      <c r="B1" s="13">
         <v>2020</v>
       </c>
-      <c r="C1" s="21">
+      <c r="C1" s="13">
         <v>2022</v>
       </c>
     </row>
@@ -1535,17 +2451,17 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" display="https://www.ferienwiki.de/feiertage/internationaler-frauentag"/>
-    <hyperlink ref="A3" r:id="rId2" display="https://www.ferienwiki.de/feiertage/tag-der-arbeit"/>
-    <hyperlink ref="A4" r:id="rId3" display="https://www.ferienwiki.de/feiertage/christi-himmelfahrt"/>
-    <hyperlink ref="A5" r:id="rId4" display="https://www.ferienwiki.de/feiertage/pfingstmontag"/>
-    <hyperlink ref="A6" r:id="rId5" display="https://www.ferienwiki.de/feiertage/fronleichnam"/>
-    <hyperlink ref="A7" r:id="rId6" display="https://www.ferienwiki.de/feiertage/maria-himmelfahrt"/>
-    <hyperlink ref="A8" r:id="rId7" display="https://www.ferienwiki.de/feiertage/weltkindertag"/>
-    <hyperlink ref="A9" r:id="rId8" display="https://www.ferienwiki.de/feiertage/tag-der-deutschen-einheit"/>
-    <hyperlink ref="A10" r:id="rId9" display="https://www.ferienwiki.de/feiertage/reformationstag"/>
-    <hyperlink ref="A11" r:id="rId10" display="https://www.ferienwiki.de/feiertage/allerheiligen"/>
-    <hyperlink ref="A12" r:id="rId11" display="https://www.ferienwiki.de/feiertage/buss-und-bettag"/>
+    <hyperlink ref="A2" r:id="rId1" display="https://www.ferienwiki.de/feiertage/internationaler-frauentag" xr:uid="{00000000-0004-0000-0300-000000000000}"/>
+    <hyperlink ref="A3" r:id="rId2" display="https://www.ferienwiki.de/feiertage/tag-der-arbeit" xr:uid="{00000000-0004-0000-0300-000001000000}"/>
+    <hyperlink ref="A4" r:id="rId3" display="https://www.ferienwiki.de/feiertage/christi-himmelfahrt" xr:uid="{00000000-0004-0000-0300-000002000000}"/>
+    <hyperlink ref="A5" r:id="rId4" display="https://www.ferienwiki.de/feiertage/pfingstmontag" xr:uid="{00000000-0004-0000-0300-000003000000}"/>
+    <hyperlink ref="A6" r:id="rId5" display="https://www.ferienwiki.de/feiertage/fronleichnam" xr:uid="{00000000-0004-0000-0300-000004000000}"/>
+    <hyperlink ref="A7" r:id="rId6" display="https://www.ferienwiki.de/feiertage/maria-himmelfahrt" xr:uid="{00000000-0004-0000-0300-000005000000}"/>
+    <hyperlink ref="A8" r:id="rId7" display="https://www.ferienwiki.de/feiertage/weltkindertag" xr:uid="{00000000-0004-0000-0300-000006000000}"/>
+    <hyperlink ref="A9" r:id="rId8" display="https://www.ferienwiki.de/feiertage/tag-der-deutschen-einheit" xr:uid="{00000000-0004-0000-0300-000007000000}"/>
+    <hyperlink ref="A10" r:id="rId9" display="https://www.ferienwiki.de/feiertage/reformationstag" xr:uid="{00000000-0004-0000-0300-000008000000}"/>
+    <hyperlink ref="A11" r:id="rId10" display="https://www.ferienwiki.de/feiertage/allerheiligen" xr:uid="{00000000-0004-0000-0300-000009000000}"/>
+    <hyperlink ref="A12" r:id="rId11" display="https://www.ferienwiki.de/feiertage/buss-und-bettag" xr:uid="{00000000-0004-0000-0300-00000A000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>